<commit_message>
benchmark: WIP fact-bank review work, saved before the lab machine closes
Uncommitted work from an earlier session (dining batch 2 edits, review
workbook and script, FACT_BANK_DECISIONS.md, fact-bank integrity test),
committed unreviewed so it survives. Affects no metric.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/review/fact_templates_review.xlsx
+++ b/docs/review/fact_templates_review.xlsx
@@ -1416,7 +1416,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">m</t>
+          <t xml:space="preserve">f</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t xml:space="preserve">{poss} पसंदीदा खाना {v} है।</t>
+          <t xml:space="preserve">{poss} पसंदीदा भोजन शैली {v} है।</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1443,13 +1443,13 @@
         <is>
           <t xml:space="preserve">f_231_dist
 My sister's favorite cuisine is South Indian.
-मेरी बहन का पसंदीदा खाना दक्षिण भारतीय है।
+मेरी बहन की पसंदीदा भोजन शैली दक्षिण भारतीय है।
 Meri sister ki favorite cuisine South Indian hai.</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t xml:space="preserve">खाना means 'food': natural for 'cuisine'? Hinglish 'cuisine' taken as f. Hindi and Hinglish nouns differ in gender here: check the Hinglish one.</t>
+          <t xml:space="preserve">Hindi uses भोजन शैली (f), not पसंदीदा खाना, because खाना ('food') overlaps favorite_dish's पकवान and the user, mother and brother have both facts: the probes must not be answerable by the other fact. Is भोजन शैली natural? Any alternative must stay distinct from पकवान. Hinglish 'cuisine' taken as f.</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">{poss} पसंदीदा खाना कौन सा है?</t>
+          <t xml:space="preserve">{poss} पसंदीदा भोजन शैली कौन सी है?</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1493,7 +1493,7 @@
         <is>
           <t xml:space="preserve">f_231_dist
 What is my sister's favorite cuisine?
-मेरी बहन का पसंदीदा खाना कौन सा है?
+मेरी बहन की पसंदीदा भोजन शैली कौन सी है?
 Meri sister ki favorite cuisine kaun si hai?</t>
         </is>
       </c>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve">एक सुधार है: {poss} पसंदीदा खाना {old} नहीं, बल्कि {new} है।</t>
+          <t xml:space="preserve">एक सुधार है: {poss} पसंदीदा भोजन शैली {old} नहीं, बल्कि {new} है।</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1538,7 +1538,7 @@
         <is>
           <t xml:space="preserve">f_233
 A correction: my brother's favorite cuisine is not Chinese, it is Bengali.
-एक सुधार है: मेरे भाई का पसंदीदा खाना चाइनीज़ नहीं, बल्कि बंगाली है।
+एक सुधार है: मेरे भाई की पसंदीदा भोजन शैली चाइनीज़ नहीं, बल्कि बंगाली है।
 Ek correction hai: mere brother ki favorite cuisine Chinese nahi, Bengali hai.</t>
         </is>
       </c>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t xml:space="preserve">अब {poss} पसंदीदा खाना कौन सा है?</t>
+          <t xml:space="preserve">अब {poss} पसंदीदा भोजन शैली कौन सी है?</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1583,7 +1583,7 @@
         <is>
           <t xml:space="preserve">f_233
 What is my brother's favorite cuisine now?
-अब मेरे भाई का पसंदीदा खाना कौन सा है?</t>
+अब मेरे भाई की पसंदीदा भोजन शैली कौन सी है?</t>
         </is>
       </c>
     </row>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Natural? Alternative: 'पेमेंट करने का मेरा पसंदीदा तरीका'.</t>
+          <t xml:space="preserve">Two का in a row ('मेरी पत्नी का पेमेंट का पसंदीदा तरीका') is grammatical, as in other relations (खेलने का पसंदीदा खेल), but is it natural? Alternatives: 'पेमेंट करने का मेरा पसंदीदा तरीका', 'पसंदीदा पेमेंट मोड'.</t>
         </is>
       </c>
     </row>
@@ -20848,9 +20848,10 @@
     <col min="3" max="3" width="26" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
     <col min="5" max="5" width="40" customWidth="1"/>
-    <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="30" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
     <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -20881,15 +20882,20 @@
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Author's note</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Verdict (OK / Fix)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Suggested fix</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Comment</t>
         </is>
@@ -20975,6 +20981,11 @@
           <t xml:space="preserve">mere father ka / mere father ki / mere father ke</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The health batch uses 'मेरे पिता' (f_101_dist); the templates use 'मेरे पिताजी'. Keep both, or align?</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -21137,6 +21148,11 @@
           <t xml:space="preserve">mere friend ka / mere friend ki / mere friend ke</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hindi 'मेरे दोस्त' / Hinglish 'mere friend' present the friend as male; English 'my friend's' is gender-neutral. Acceptable, or use a fixed-gender person?</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -21247,9 +21263,9 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H14"/>
+  <autoFilter ref="A1:I14"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F14">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G14">
       <formula1>"OK,Fix"</formula1>
     </dataValidation>
   </dataValidations>
@@ -24804,7 +24820,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grammar: 'मेरी अगली महीने मनाली जाने की योजना है।' Expected: 'अगले महीने मेरी मनाली जाने की योजना है।'. Not fixed: the Sep pilot used it.</t>
+          <t xml:space="preserve">Grammar: 'मेरी अगली महीने मनाली जाने की योजना है।' Proposed: 'अगले महीने मेरी मनाली जाने की योजना है।' (महीना is m: अगले महीने).</t>
         </is>
       </c>
     </row>
@@ -24821,12 +24837,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">f_002, f_003, f_004, f_008, f_009, f_012, f_017</t>
+          <t xml:space="preserve">f_006</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hindi uses masculine speaker verbs ('रहता हूँ', 'करता हूँ'). The new templates avoid speaker gender. Rewrite these, or document the speaker as male?</t>
+          <t xml:space="preserve">Question drops 'morning', which the fact needs ('favorite MORNING beverage'), and the Hindi has a gender error ('मेरी पसंदीदा पेय': पेय is m). Proposed: en 'What is my favorite morning beverage?', hi 'सुबह की मेरी पसंदीदा ड्रिंक क्या है?' (ड्रिंक as in the statement), hi-en 'Meri favorite morning beverage kya hai?' (matches the statement's 'Meri').</t>
         </is>
       </c>
     </row>
@@ -24838,24 +24854,90 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t xml:space="preserve">facts_v1.yaml, health_batch_01.yaml</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f_002, f_003, f_004, f_008, f_009, f_012, f_017; f_103, f_104, f_104_dist, f_106, f_109, f_110</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-person verbs are masculine ('रहता हूँ', 'karta hoon'). Grammatical for a male speaker (BENCHMARK_SPEC §7.2 uses 'मैं पुणे में रहता हूँ'), so this is a speaker-persona question, not an error. The templates avoid first-person verbs entirely. Decide: document a male speaker, or rewrite these without speaker gender.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">health_batch_01.yaml, facts_v1.yaml</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f_104, f_104_dist, f_012</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overlapping diet facts for the user. f_104_dist (vegetarian, 'I am also vegetarian') restates f_012 (vegetarian, 'I follow a strictly vegetarian diet') under another relation name. f_104's question 'What kind of diet do I follow?' is also answered by f_012; both are base facts, so both are asked. (f_104_dist shares f_104's question, as a value-shift distractor does, but distractors are never asked.) Needs a decision (docs/review/FACT_BANK_DECISIONS.md, item A); not changed here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">facts_v1.yaml</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f_004</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">domain is 'languages', which is not one of the 8 approved domains (BENCHMARK_SPEC §3). Which domain should it count under?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t xml:space="preserve">health_batch_01.yaml</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">f_104_dist</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(user, dietary_restriction, vegetarian) is the same fact as facts_v1 f_012 (user, dietary_preference, vegetarian). Drop one before merging.</t>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f_105, f_109, f_110</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value keys (flu_shot_pending, regular_donor, yoga_daily) are abstract labels that occur in none of the sentences, and hand-written facts have no value_aliases. Today strict matching can credit them only when a memory contains a whole authored sentence verbatim; a paraphrase never matches. Which aliases are authorized is decision D1.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A1:G7"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="E2:E4">
+    <dataValidation type="list" allowBlank="1" sqref="E2:E7">
       <formula1>"OK,Fix"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>